<commit_message>
modul 1 test version 1 klar
</commit_message>
<xml_diff>
--- a/hojatimmar.xlsx
+++ b/hojatimmar.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alias\Documents\Projekt\hoja\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4690DCDA-5439-4E32-879E-23EBFF74F7BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4542EA0D-2C88-4FC6-9FD4-C3D61C3C5792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4B11DD80-208B-418E-BD56-3D5666C184EF}"/>
+    <workbookView xWindow="7200" yWindow="1545" windowWidth="11820" windowHeight="11385" xr2:uid="{4B11DD80-208B-418E-BD56-3D5666C184EF}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -755,8 +755,12 @@
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="2"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="9"/>
+      <c r="C20" s="5">
+        <v>44802</v>
+      </c>
+      <c r="D20" s="9">
+        <v>0.26041666666666669</v>
+      </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="2"/>
@@ -829,11 +833,11 @@
       </c>
       <c r="C34" s="16">
         <f ca="1">TODAY()</f>
-        <v>44801</v>
+        <v>44802</v>
       </c>
       <c r="D34" s="18">
         <f>SUM(D7:D32)</f>
-        <v>1.3298611111111109</v>
+        <v>1.5902777777777777</v>
       </c>
     </row>
     <row r="35" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>